<commit_message>
End-of-semester: cheat sheet, group final, May email draft
Final pre-archival commit before this repo retires:
- cheat-sheet.md: condensed exam reference distilled from course-notes
- modules/module-14/group-assignment/: final report PDF + presentation video
- resources/email-drafts.md: added May 2026 follow-up to Griffiths re:
  August grad submissions before paternal leave
- resources/ME_Plan_of_Study_Worksheet.xlsx: worksheet updates

Graduation materials (email-drafts, plan-of-study worksheet, etc.) have
been migrated to laws-smith-luna/homework. This repo will be archived
after this commit.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/ME_Plan_of_Study_Worksheet.xlsx
+++ b/resources/ME_Plan_of_Study_Worksheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lawss\Documents\Repos\User Interface Design\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA02C3C3-60F5-487E-B86C-DCEE88792414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E810703B-FBE2-47DE-B039-E1E9A2E1E415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{6C2D3FD5-6A10-44FA-9DBD-AC6BD9D1CEE9}"/>
   </bookViews>
@@ -877,7 +877,7 @@
         <v>1</v>
       </c>
       <c r="J3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" s="2">
         <v>0</v>
@@ -910,7 +910,7 @@
         <v>1</v>
       </c>
       <c r="J4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="2">
         <v>0</v>
@@ -943,7 +943,7 @@
         <v>1</v>
       </c>
       <c r="J5" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="2">
         <v>0</v>
@@ -976,7 +976,7 @@
         <v>1</v>
       </c>
       <c r="J6" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="2">
         <v>0</v>
@@ -1011,7 +1011,7 @@
         <v>1</v>
       </c>
       <c r="J7" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K7" s="2">
         <v>0</v>
@@ -1044,7 +1044,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" s="2">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>0</v>
       </c>
       <c r="J9" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" s="2">
         <v>0</v>
@@ -1108,7 +1108,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10" s="2">
         <v>0</v>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="J11" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" s="2">
         <v>0</v>
@@ -1197,12 +1197,8 @@
         <v>47</v>
       </c>
       <c r="H13" s="2"/>
-      <c r="I13" s="2">
-        <v>1</v>
-      </c>
-      <c r="J13" s="2">
-        <v>1</v>
-      </c>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
       <c r="K13" s="2">
         <v>0</v>
       </c>
@@ -1260,11 +1256,11 @@
       </c>
       <c r="B19" s="2">
         <f>SUMPRODUCT(F3:F15,I3:I15)</f>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C19" s="2" t="str">
         <f>IF(B19&lt;18,"Not Satisfied","Satisfied")</f>
-        <v>Satisfied</v>
+        <v>Not Satisfied</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
@@ -1273,11 +1269,11 @@
       </c>
       <c r="B20" s="2">
         <f>SUMPRODUCT(F3:F15,J3:J15)</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C20" s="2" t="str">
         <f>IF(B20&gt;9,"Not Satisfied","Satisfied")</f>
-        <v>Not Satisfied</v>
+        <v>Satisfied</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
@@ -1286,11 +1282,11 @@
       </c>
       <c r="B21" s="2">
         <f>SUMPRODUCT(F3:F15,I3:I15,J3:J15)</f>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="C21" s="2" t="str">
         <f>IF(B21&gt;6,"Not Satisfied","Satisfied")</f>
-        <v>Not Satisfied</v>
+        <v>Satisfied</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>